<commit_message>
edited project proposal latex: added role
</commit_message>
<xml_diff>
--- a/timesheets/Nina.xlsx
+++ b/timesheets/Nina.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\wu_dslab_infrared-city\timesheets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{527A64EE-2652-4509-BBD5-661975FC3197}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BA57D73-55EB-4EB9-8A7F-522F8FCF1099}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="27900" yWindow="11880" windowWidth="15024" windowHeight="11856" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="7080" yWindow="10236" windowWidth="15024" windowHeight="11856" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>Date</t>
   </si>
@@ -56,7 +56,10 @@
     <t>researched use of Vienna Baumkataster datasets, defined data coach questions, wrote meeting protocol</t>
   </si>
   <si>
-    <t>finalized meeting protocol, pushed protocol and latex template on github</t>
+    <t>finalized and pushed meeting protocol on github</t>
+  </si>
+  <si>
+    <t>pushed latex project proposal changes on github</t>
   </si>
 </sst>
 </file>
@@ -375,7 +378,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13.21875" customWidth="1"/>
@@ -431,7 +434,18 @@
         <v>6</v>
       </c>
       <c r="C4">
-        <v>1</v>
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A5" s="1">
+        <v>46092</v>
+      </c>
+      <c r="B5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5">
+        <v>0.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
edited nina timesheet 12.03.26
</commit_message>
<xml_diff>
--- a/timesheets/Nina.xlsx
+++ b/timesheets/Nina.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\wu_dslab_infrared-city\timesheets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BA57D73-55EB-4EB9-8A7F-522F8FCF1099}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40644C24-859A-4DCF-92DD-DFBC43E66008}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7080" yWindow="10236" windowWidth="15024" windowHeight="11856" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6996" yWindow="9672" windowWidth="20136" windowHeight="14976" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
   <si>
     <t>Date</t>
   </si>
@@ -60,6 +60,9 @@
   </si>
   <si>
     <t>pushed latex project proposal changes on github</t>
+  </si>
+  <si>
+    <t>finalized data coach questions and pushed on github for meeting</t>
   </si>
 </sst>
 </file>
@@ -378,7 +381,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13.21875" customWidth="1"/>
@@ -412,7 +415,7 @@
       </c>
       <c r="H2">
         <f>SUM(C:C)</f>
-        <v>7</v>
+        <v>8.5</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -446,6 +449,17 @@
       </c>
       <c r="C5">
         <v>0.5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A6" s="1">
+        <v>46093</v>
+      </c>
+      <c r="B6" t="s">
+        <v>8</v>
+      </c>
+      <c r="C6">
+        <v>1.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added meeting protocol of 26.03 and edit timesheet
</commit_message>
<xml_diff>
--- a/timesheets/Nina.xlsx
+++ b/timesheets/Nina.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\wu_dslab_infrared-city\timesheets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B857AE78-209C-4C34-867B-AB9AED2F4C44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABAD18D1-6E72-4192-B688-F81480D20E39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="15204" yWindow="11088" windowWidth="19008" windowHeight="11856" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
   <si>
     <t>Date</t>
   </si>
@@ -78,6 +78,9 @@
   </si>
   <si>
     <t>making juypter notebook file + starting writing scraper code</t>
+  </si>
+  <si>
+    <t>finalized and pushed new meeting protocol on github</t>
   </si>
 </sst>
 </file>
@@ -312,7 +315,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13.21875" customWidth="1"/>
@@ -346,7 +349,7 @@
       </c>
       <c r="H2">
         <f>SUM(C:C)</f>
-        <v>16</v>
+        <v>16.5</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -446,6 +449,17 @@
       </c>
       <c r="C11">
         <v>2.5</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A12" s="1">
+        <v>46104</v>
+      </c>
+      <c r="B12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C12">
+        <v>0.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
edited timesheet nina 25.0326
</commit_message>
<xml_diff>
--- a/timesheets/Nina.xlsx
+++ b/timesheets/Nina.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\wu_dslab_infrared-city\timesheets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABAD18D1-6E72-4192-B688-F81480D20E39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F1212C8-5500-43B5-9CC8-80CD8F053F24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="15204" yWindow="11088" windowWidth="19008" windowHeight="11856" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="13128" yWindow="11592" windowWidth="19008" windowHeight="11856" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
   <si>
     <t>Date</t>
   </si>
@@ -81,6 +81,9 @@
   </si>
   <si>
     <t>finalized and pushed new meeting protocol on github</t>
+  </si>
+  <si>
+    <t>continued wiht scraper code + foudn new datasets</t>
   </si>
 </sst>
 </file>
@@ -315,7 +318,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13.21875" customWidth="1"/>
@@ -349,7 +352,7 @@
       </c>
       <c r="H2">
         <f>SUM(C:C)</f>
-        <v>16.5</v>
+        <v>18</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -460,6 +463,17 @@
       </c>
       <c r="C12">
         <v>0.5</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A13" s="1">
+        <v>46106</v>
+      </c>
+      <c r="B13" t="s">
+        <v>15</v>
+      </c>
+      <c r="C13">
+        <v>1.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
edited nina timesheet 7.5.26
</commit_message>
<xml_diff>
--- a/timesheets/Nina.xlsx
+++ b/timesheets/Nina.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vani1\wu_dslab_infrared-city\timesheets\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vani1\Desktop\wu_dslab_infrared-city\timesheets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4857272-7B1D-4C2E-9DEB-9144F0E9A690}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E44A20C-6020-4C2A-8C94-FEE4791FC16D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10560" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
   <si>
     <t>Date</t>
   </si>
@@ -110,13 +110,22 @@
     <t>finalized notebooks (added descriptions, etc.)</t>
   </si>
   <si>
-    <t>fixing typos in notebooks</t>
-  </si>
-  <si>
     <t>starting writing scraper for sentinel/osm -&gt; explored the option of automating copernicus sentinel 2 API -&gt; didnt work so well</t>
   </si>
   <si>
     <t>wrote two meeting protocols and discussed EDA outcome with sara (no rescraping necessary)</t>
+  </si>
+  <si>
+    <t>scraped osm data and satellite data for Innsbruck and Linz</t>
+  </si>
+  <si>
+    <t>fixing typos in notebooks and finialzed my chapter for intermediate report</t>
+  </si>
+  <si>
+    <t>wrote sparring group protocol for my group: suggestions, feedback etc.</t>
+  </si>
+  <si>
+    <t>scraped more baumkataster datasets for Innsbruck and Linz</t>
   </si>
 </sst>
 </file>
@@ -351,7 +360,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H24"/>
+  <dimension ref="A1:H27"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="13.1796875" customWidth="1"/>
@@ -385,7 +394,7 @@
       </c>
       <c r="H2">
         <f>SUM(C:C)</f>
-        <v>47</v>
+        <v>60</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.35">
@@ -569,7 +578,7 @@
         <v>46111</v>
       </c>
       <c r="B19" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C19">
         <v>3</v>
@@ -613,10 +622,10 @@
         <v>46113</v>
       </c>
       <c r="B23" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="C23">
-        <v>0.5</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.35">
@@ -624,10 +633,43 @@
         <v>46125</v>
       </c>
       <c r="B24" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C24">
         <v>0.5</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A25" s="1">
+        <v>46086</v>
+      </c>
+      <c r="B25" t="s">
+        <v>28</v>
+      </c>
+      <c r="C25">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A26" s="1">
+        <v>46148</v>
+      </c>
+      <c r="B26" t="s">
+        <v>29</v>
+      </c>
+      <c r="C26">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A27" s="1">
+        <v>46149</v>
+      </c>
+      <c r="B27" t="s">
+        <v>26</v>
+      </c>
+      <c r="C27">
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
edited timesheet for 30-526
</commit_message>
<xml_diff>
--- a/timesheets/Nina.xlsx
+++ b/timesheets/Nina.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vani1\Desktop\wu_dslab_infrared-city\timesheets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{897CF734-29C3-4869-B769-BFCE9710992E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{600F84E2-ADBB-4EAF-AA4D-73E65E933568}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10560" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="34">
   <si>
     <t>Date</t>
   </si>
@@ -135,6 +135,9 @@
   </si>
   <si>
     <t>scraped sentinel-2 data for 5 cities (3 seasons again), adjusted BEAM again, wrote chapters for Draft Report &amp; Slides</t>
+  </si>
+  <si>
+    <t>finished my chapters and fixed Draft BEAM</t>
   </si>
 </sst>
 </file>
@@ -369,7 +372,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H30"/>
+  <dimension ref="A1:H31"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="13.1796875" customWidth="1"/>
@@ -403,7 +406,7 @@
       </c>
       <c r="H2">
         <f>SUM(C:C)</f>
-        <v>80</v>
+        <v>82</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.35">
@@ -712,6 +715,17 @@
       </c>
       <c r="C30">
         <v>6</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A31" s="1">
+        <v>46172</v>
+      </c>
+      <c r="B31" t="s">
+        <v>33</v>
+      </c>
+      <c r="C31">
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>